<commit_message>
feat: setup complete Appium WDIO TypeScript automation testing framework and GHA Summary dashboard integration
</commit_message>
<xml_diff>
--- a/tests/test_report.xlsx
+++ b/tests/test_report.xlsx
@@ -558,7 +558,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18 11:07:02</t>
+          <t>2026-06-18 14:53:31</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Interview Session</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.011</v>
+        <v>0.012</v>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Candidate Analytics</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="F11" s="11" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Histories &amp; Logs</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Histories &amp; Logs</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="F15" s="11" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
@@ -931,7 +931,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Histories &amp; Logs</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="F16" s="8" t="n">
-        <v>0.011</v>
+        <v>0.012</v>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
@@ -966,7 +966,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Interview Session</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -980,7 +980,7 @@
         </is>
       </c>
       <c r="F17" s="11" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Interview Session</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Interview Session</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Interview Session</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Interview Session</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1120,7 +1120,7 @@
         </is>
       </c>
       <c r="F21" s="11" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Evaluation Results</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Evaluation Results</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Evaluation Results</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="F24" s="8" t="n">
-        <v>0.011</v>
+        <v>0.012</v>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Resume Analyzer</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="F25" s="11" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Resume Analyzer</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Interview Session</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Interview Session</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Interview Session</t>
+          <t>Mobile Features</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="F33" s="11" t="n">
-        <v>0.021</v>
+        <v>0.022</v>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
@@ -1645,7 +1645,7 @@
         </is>
       </c>
       <c r="F36" s="8" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1680,7 +1680,7 @@
         </is>
       </c>
       <c r="F37" s="11" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Landing Page</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="F39" s="11" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Landing Page</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Histories &amp; Logs</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="F44" s="8" t="n">
-        <v>0.021</v>
+        <v>0.023</v>
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -1960,7 +1960,7 @@
         </is>
       </c>
       <c r="F45" s="11" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="F46" s="8" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Evaluation Results</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Interview Session</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="F48" s="8" t="n">
-        <v>0.023</v>
+        <v>0.022</v>
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -2100,7 +2100,7 @@
         </is>
       </c>
       <c r="F49" s="11" t="n">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="F52" s="8" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -2240,7 +2240,7 @@
         </is>
       </c>
       <c r="F53" s="11" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Candidate Analytics</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="F55" s="11" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="F56" s="8" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Mobile Navigation</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -2380,7 +2380,7 @@
         </is>
       </c>
       <c r="F57" s="11" t="n">
-        <v>0.011</v>
+        <v>0.012</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
@@ -2450,7 +2450,7 @@
         </is>
       </c>
       <c r="F59" s="11" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="F60" s="8" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
@@ -2520,7 +2520,7 @@
         </is>
       </c>
       <c r="F61" s="11" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="F62" s="8" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -2660,7 +2660,7 @@
         </is>
       </c>
       <c r="F65" s="11" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
@@ -2695,7 +2695,7 @@
         </is>
       </c>
       <c r="F66" s="8" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2730,7 +2730,7 @@
         </is>
       </c>
       <c r="F67" s="11" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
@@ -2765,7 +2765,7 @@
         </is>
       </c>
       <c r="F68" s="8" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -2800,7 +2800,7 @@
         </is>
       </c>
       <c r="F69" s="11" t="n">
-        <v>0.011</v>
+        <v>0.012</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -2870,7 +2870,7 @@
         </is>
       </c>
       <c r="F71" s="11" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2940,7 +2940,7 @@
         </is>
       </c>
       <c r="F73" s="11" t="n">
-        <v>0.039</v>
+        <v>0.038</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -3010,7 +3010,7 @@
         </is>
       </c>
       <c r="F75" s="11" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
@@ -3045,7 +3045,7 @@
         </is>
       </c>
       <c r="F76" s="8" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -3171,7 +3171,7 @@
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
@@ -3255,7 +3255,7 @@
         </is>
       </c>
       <c r="F82" s="8" t="n">
-        <v>0.017</v>
+        <v>0.016</v>
       </c>
       <c r="G82" s="9" t="inlineStr">
         <is>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="F84" s="8" t="n">
-        <v>0.043</v>
+        <v>0.045</v>
       </c>
       <c r="G84" s="9" t="inlineStr">
         <is>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -3395,7 +3395,7 @@
         </is>
       </c>
       <c r="F86" s="8" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="G86" s="9" t="inlineStr">
         <is>
@@ -3416,7 +3416,7 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="C88" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
@@ -3465,7 +3465,7 @@
         </is>
       </c>
       <c r="F88" s="8" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="G88" s="9" t="inlineStr">
         <is>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -3535,7 +3535,7 @@
         </is>
       </c>
       <c r="F90" s="8" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="G90" s="9" t="inlineStr">
         <is>
@@ -3556,7 +3556,7 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -3591,7 +3591,7 @@
       </c>
       <c r="C92" s="9" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="F92" s="8" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="G92" s="9" t="inlineStr">
         <is>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -3640,7 +3640,7 @@
         </is>
       </c>
       <c r="F93" s="11" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="C94" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
@@ -3710,7 +3710,7 @@
         </is>
       </c>
       <c r="F95" s="11" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -3815,7 +3815,7 @@
         </is>
       </c>
       <c r="F98" s="8" t="n">
-        <v>0.017</v>
+        <v>0.019</v>
       </c>
       <c r="G98" s="9" t="inlineStr">
         <is>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="C100" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
@@ -3885,7 +3885,7 @@
         </is>
       </c>
       <c r="F100" s="8" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="G100" s="9" t="inlineStr">
         <is>
@@ -3920,7 +3920,7 @@
         </is>
       </c>
       <c r="F101" s="11" t="n">
-        <v>0.017</v>
+        <v>0.016</v>
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
@@ -3990,7 +3990,7 @@
         </is>
       </c>
       <c r="F103" s="11" t="n">
-        <v>0.017</v>
+        <v>0.016</v>
       </c>
       <c r="G103" s="4" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -4130,7 +4130,7 @@
         </is>
       </c>
       <c r="F107" s="11" t="n">
-        <v>0.011</v>
+        <v>0.012</v>
       </c>
       <c r="G107" s="4" t="inlineStr">
         <is>
@@ -4200,7 +4200,7 @@
         </is>
       </c>
       <c r="F109" s="11" t="n">
-        <v>0.023</v>
+        <v>0.022</v>
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="C110" s="9" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D110" s="9" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="C112" s="9" t="inlineStr">
         <is>
-          <t>Dashboard / Sidebar</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D112" s="9" t="inlineStr">
@@ -4305,7 +4305,7 @@
         </is>
       </c>
       <c r="F112" s="8" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="G112" s="9" t="inlineStr">
         <is>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -4340,7 +4340,7 @@
         </is>
       </c>
       <c r="F113" s="11" t="n">
-        <v>0.017</v>
+        <v>0.016</v>
       </c>
       <c r="G113" s="4" t="inlineStr">
         <is>
@@ -4375,7 +4375,7 @@
         </is>
       </c>
       <c r="F114" s="8" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="G114" s="9" t="inlineStr">
         <is>
@@ -4396,7 +4396,7 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>General System</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">

</xml_diff>